<commit_message>
sort button on crm page s.no
</commit_message>
<xml_diff>
--- a/results_backup.xlsx
+++ b/results_backup.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z125"/>
+  <dimension ref="A1:Z126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="28.33203125" customWidth="1" min="3" max="3"/>
@@ -604,7 +604,11 @@
   <sheetData>
     <row r="1" ht="17" customFormat="1" customHeight="1" s="9">
       <c r="A1" s="7" t="n"/>
-      <c r="B1" s="7" t="n"/>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Company</t>
@@ -979,22 +983,23 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2026_x000D__x000D_
-Apr 17 - call fedex for haribabu laptop_x000D__x000D_
-Jun 12 - WA - hello_x000D__x000D_
-Jun 23 - WA - are you on paternity leave?_x000D__x000D_
-Jul 1 - WA call - did not receive_x000D__x000D_
-Jul 13 - WA Hello - No response_x000D__x000D_
-Jul 21 - WA Hello - No response_x000D__x000D_
-Jul 24 - WA resonded - was busy_x000D__x000D_
-Jul 27 - call - he asked to be patient. Will let me know who to move forward with Kirti_x000D__x000D_
-Aug 10 - call - he had no clue what happening._x000D__x000D_
-Aug 27 - WA - any info found out?_x000D__x000D_
-Aug 31 - called BBC can now work with anyone via MBO_x000D__x000D_
-Sep 2 - WA How to reach out to kiriti_x000D__x000D_
-Sep 14-16 - lets connect_x000D__x000D_
-Sep 22 - Lets connect_x000D_
-Sep 23 - Called will share the MDs who are doing large business that i cn ask DD to introduce</t>
+          <t>2026
+Apr 17 - call fedex for haribabu laptop
+Jun 12 - WA - hello
+Jun 23 - WA - are you on paternity leave?
+Jul 1 - WA call - did not receive
+Jul 13 - WA Hello - No response
+Jul 21 - WA Hello - No response
+Jul 24 - WA resonded - was busy
+Jul 27 - call - he asked to be patient. Will let me know who to move forward with Kirti
+Aug 10 - call - he had no clue what happening.
+Aug 27 - WA - any info found out?
+Aug 31 - called BBC can now work with anyone via MBO
+Sep 2 - WA How to reach out to kiriti
+Sep 14-16 - lets connect
+Sep 22 - Lets connect
+Sep 23 - Called will share the MDs who are doing large business that i cn ask DD to introduce
+Oct 9 - Met in person in ATL</t>
         </is>
       </c>
       <c r="F9" s="1" t="n"/>
@@ -1781,7 +1786,12 @@
           <t>Bobby Karer - US Cold Storage</t>
         </is>
       </c>
-      <c r="E27" s="1" t="n"/>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>2026
+Sep 26 - No hiring now</t>
+        </is>
+      </c>
       <c r="F27" s="1" t="n"/>
       <c r="G27" s="1" t="n"/>
       <c r="H27" s="1" t="n"/>
@@ -5883,10 +5893,8 @@
       <c r="Z121" s="1" t="n"/>
     </row>
     <row r="122">
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>121</t>
-        </is>
+      <c r="B122" s="1" t="n">
+        <v>121</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -5906,10 +5914,8 @@
       </c>
     </row>
     <row r="123">
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>117</t>
-        </is>
+      <c r="B123" s="1" t="n">
+        <v>122</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -5929,10 +5935,8 @@
       </c>
     </row>
     <row r="124">
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>122</t>
-        </is>
+      <c r="B124" s="1" t="n">
+        <v>123</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -5952,11 +5956,8 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="B125" s="1" t="n">
+        <v>124</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
@@ -5974,27 +5975,29 @@
 Oct 19 - meeting at Ravi;s card party from Meghalaya, has body shop and PA and NJ state client</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
-      <c r="O125" t="inlineStr"/>
-      <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr"/>
-      <c r="R125" t="inlineStr"/>
-      <c r="S125" t="inlineStr"/>
-      <c r="T125" t="inlineStr"/>
-      <c r="U125" t="inlineStr"/>
-      <c r="V125" t="inlineStr"/>
-      <c r="W125" t="inlineStr"/>
-      <c r="X125" t="inlineStr"/>
-      <c r="Y125" t="inlineStr"/>
-      <c r="Z125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Tushar Tanpure,  recruiter , Pune</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2026
+Oct 22- email for F/T req check</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -10058,7 +10061,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I118"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -15392,7 +15395,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L95"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -19446,7 +19449,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -20011,7 +20014,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>